<commit_message>
update: add keyboard feet, update CAD models, update BOM
</commit_message>
<xml_diff>
--- a/Hardware/bom/bom.xlsx
+++ b/Hardware/bom/bom.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ritam\Documents\projects\hardware\sheaf65\Hardware\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D41B843E-0D94-42B3-8649-A51A772519B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20F7D77E-BC7C-4C82-84F6-16104E8AA1DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{7EBACB66-221B-455C-9668-D99D7DBAA942}"/>
   </bookViews>
   <sheets>
     <sheet name="bom" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="73">
   <si>
     <t>Category</t>
   </si>
@@ -212,6 +225,33 @@
   </si>
   <si>
     <t>https://onlyscrews.in/products/m2-x-8mm-phillips-round-head-laptop-screw-1</t>
+  </si>
+  <si>
+    <t>Threaded Insert</t>
+  </si>
+  <si>
+    <t>M4 x 4mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M4 x 8mm </t>
+  </si>
+  <si>
+    <t>https://onlyscrews.in/products/m4-x-4mm-brass-threaded-inserts-2</t>
+  </si>
+  <si>
+    <t>https://onlyscrews.in/products/phillips-pan-head-m4-x-8mm-pack-of-20</t>
+  </si>
+  <si>
+    <t>Plate, Backplate</t>
+  </si>
+  <si>
+    <t>Rubber Feet</t>
+  </si>
+  <si>
+    <t>8mm Self Adhesive</t>
+  </si>
+  <si>
+    <t>https://www.amazon.in/Miramar-Adhesive-Non-Slip-Furniture-Hemispherical/dp/B0BLN4TCPT</t>
   </si>
 </sst>
 </file>
@@ -1073,7 +1113,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FFEDD07-4F54-47C1-AF97-745393103FF2}">
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
@@ -1156,7 +1196,7 @@
         <v>96</v>
       </c>
       <c r="G3" t="str">
-        <f t="shared" ref="G3:G18" si="0">_xlfn.CONCAT("~$",ROUND(F3/93, 2))</f>
+        <f t="shared" ref="G3:G13" si="0">_xlfn.CONCAT("~$",ROUND(F3/93, 2))</f>
         <v>~$1.03</v>
       </c>
       <c r="H3" t="s">
@@ -1384,26 +1424,26 @@
         <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C12" t="s">
-        <v>41</v>
+        <v>66</v>
       </c>
       <c r="D12" t="s">
         <v>36</v>
       </c>
       <c r="E12">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="F12">
-        <v>56</v>
+        <v>4.4000000000000004</v>
       </c>
       <c r="G12" t="str">
         <f t="shared" si="0"/>
-        <v>~$0.6</v>
+        <v>~$0.05</v>
       </c>
       <c r="H12" t="s">
-        <v>42</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1411,10 +1451,10 @@
         <v>33</v>
       </c>
       <c r="B13" t="s">
-        <v>40</v>
+        <v>64</v>
       </c>
       <c r="C13" t="s">
-        <v>43</v>
+        <v>65</v>
       </c>
       <c r="D13" t="s">
         <v>36</v>
@@ -1423,135 +1463,217 @@
         <v>2</v>
       </c>
       <c r="F13">
-        <v>8</v>
+        <v>6.4</v>
       </c>
       <c r="G13" t="str">
         <f t="shared" si="0"/>
-        <v>~$0.09</v>
+        <v>~$0.07</v>
       </c>
       <c r="H13" t="s">
-        <v>44</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="B14" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C14" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="D14" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="E14">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="G14" t="str">
-        <f t="shared" si="0"/>
-        <v>~$0</v>
+        <f>_xlfn.CONCAT("~$",ROUND(F14/93, 2))</f>
+        <v>~$0.6</v>
+      </c>
+      <c r="H14" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
       <c r="B15" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="C15" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="D15" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="E15">
-        <v>70</v>
-      </c>
-      <c r="F15" s="1">
-        <v>1680</v>
+        <v>2</v>
+      </c>
+      <c r="F15">
+        <v>8</v>
       </c>
       <c r="G15" t="str">
-        <f t="shared" si="0"/>
-        <v>~$18.06</v>
+        <f>_xlfn.CONCAT("~$",ROUND(F15/93, 2))</f>
+        <v>~$0.09</v>
       </c>
       <c r="H15" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B16" t="s">
-        <v>53</v>
+        <v>70</v>
       </c>
       <c r="C16" t="s">
-        <v>54</v>
+        <v>71</v>
       </c>
       <c r="D16" t="s">
-        <v>55</v>
+        <v>11</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="F16">
-        <v>1800</v>
+        <v>189</v>
       </c>
       <c r="G16" t="str">
-        <f t="shared" si="0"/>
-        <v>~$19.35</v>
+        <f>_xlfn.CONCAT("~$",ROUND(F16/93, 2))</f>
+        <v>~$2.03</v>
       </c>
       <c r="H16" t="s">
-        <v>56</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B17" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="C17" t="s">
-        <v>58</v>
+        <v>46</v>
       </c>
       <c r="D17" t="s">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="E17">
         <v>1</v>
       </c>
       <c r="F17">
-        <v>380</v>
+        <v>0</v>
       </c>
       <c r="G17" t="str">
-        <f t="shared" si="0"/>
-        <v>~$4.09</v>
-      </c>
-      <c r="H17" t="s">
-        <v>60</v>
+        <f>_xlfn.CONCAT("~$",ROUND(F17/93, 2))</f>
+        <v>~$0</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" t="s">
+        <v>50</v>
+      </c>
+      <c r="D18" t="s">
+        <v>51</v>
+      </c>
+      <c r="E18">
+        <v>70</v>
+      </c>
+      <c r="F18" s="1">
+        <v>1680</v>
+      </c>
+      <c r="G18" t="str">
+        <f>_xlfn.CONCAT("~$",ROUND(F18/93, 2))</f>
+        <v>~$18.06</v>
+      </c>
+      <c r="H18" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" t="s">
+        <v>54</v>
+      </c>
+      <c r="D19" t="s">
+        <v>55</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19">
+        <v>1800</v>
+      </c>
+      <c r="G19" t="str">
+        <f>_xlfn.CONCAT("~$",ROUND(F19/93, 2))</f>
+        <v>~$19.35</v>
+      </c>
+      <c r="H19" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>48</v>
+      </c>
+      <c r="B20" t="s">
+        <v>57</v>
+      </c>
+      <c r="C20" t="s">
+        <v>58</v>
+      </c>
+      <c r="D20" t="s">
+        <v>59</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20">
+        <v>380</v>
+      </c>
+      <c r="G20" t="str">
+        <f>_xlfn.CONCAT("~$",ROUND(F20/93, 2))</f>
+        <v>~$4.09</v>
+      </c>
+      <c r="H20" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>61</v>
       </c>
-      <c r="F18">
-        <f>SUM(F2:F17)</f>
-        <v>10089.6</v>
-      </c>
-      <c r="G18" t="str">
-        <f t="shared" si="0"/>
-        <v>~$108.49</v>
+      <c r="F21">
+        <f>SUM(F2:F20)</f>
+        <v>10289.4</v>
+      </c>
+      <c r="G21" t="str">
+        <f>_xlfn.CONCAT("~$",ROUND(F21/93, 2))</f>
+        <v>~$110.64</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
TTC PY V2 hotswap sockets
</commit_message>
<xml_diff>
--- a/Hardware/bom/bom.xlsx
+++ b/Hardware/bom/bom.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ritam\Documents\projects\hardware\sheaf65\Hardware\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20F7D77E-BC7C-4C82-84F6-16104E8AA1DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40B49539-CAB5-4DC5-A14E-534487C5468A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{7EBACB66-221B-455C-9668-D99D7DBAA942}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="74">
   <si>
     <t>Category</t>
   </si>
@@ -113,12 +113,6 @@
     <t>Hotswap Socket</t>
   </si>
   <si>
-    <t>SMD Hotswap Socket</t>
-  </si>
-  <si>
-    <t>Kailh</t>
-  </si>
-  <si>
     <t>https://meckeys.com/shop/accessories/keyboard-accessories/key-switches/kailh-hot-swap-socket/</t>
   </si>
   <si>
@@ -252,6 +246,15 @@
   </si>
   <si>
     <t>https://www.amazon.in/Miramar-Adhesive-Non-Slip-Furniture-Hemispherical/dp/B0BLN4TCPT</t>
+  </si>
+  <si>
+    <t>TTC</t>
+  </si>
+  <si>
+    <t>TTC Pokayoke V2 Socket</t>
+  </si>
+  <si>
+    <t>Shipping</t>
   </si>
 </sst>
 </file>
@@ -1113,7 +1116,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FFEDD07-4F54-47C1-AF97-745393103FF2}">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
@@ -1292,23 +1295,23 @@
         <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="D7" t="s">
-        <v>27</v>
+        <v>71</v>
       </c>
       <c r="E7">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F7">
-        <v>532</v>
+        <v>680</v>
       </c>
       <c r="G7" t="str">
         <f t="shared" si="0"/>
-        <v>~$5.72</v>
+        <v>~$7.31</v>
       </c>
       <c r="H7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1316,13 +1319,13 @@
         <v>8</v>
       </c>
       <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" t="s">
         <v>29</v>
-      </c>
-      <c r="C8" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" t="s">
-        <v>31</v>
       </c>
       <c r="E8">
         <v>5</v>
@@ -1335,21 +1338,21 @@
         <v>~$51.61</v>
       </c>
       <c r="H8" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
         <v>33</v>
       </c>
-      <c r="B9" t="s">
+      <c r="D9" t="s">
         <v>34</v>
-      </c>
-      <c r="C9" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9" t="s">
-        <v>36</v>
       </c>
       <c r="E9">
         <v>2</v>
@@ -1362,21 +1365,21 @@
         <v>~$0.08</v>
       </c>
       <c r="H9" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" t="s">
         <v>34</v>
-      </c>
-      <c r="C10" t="s">
-        <v>38</v>
-      </c>
-      <c r="D10" t="s">
-        <v>36</v>
       </c>
       <c r="E10">
         <v>12</v>
@@ -1389,21 +1392,21 @@
         <v>~$0.52</v>
       </c>
       <c r="H10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B11" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" t="s">
+        <v>60</v>
+      </c>
+      <c r="D11" t="s">
         <v>34</v>
-      </c>
-      <c r="C11" t="s">
-        <v>62</v>
-      </c>
-      <c r="D11" t="s">
-        <v>36</v>
       </c>
       <c r="E11">
         <v>10</v>
@@ -1416,21 +1419,21 @@
         <v>~$0.47</v>
       </c>
       <c r="H11" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" t="s">
+        <v>64</v>
+      </c>
+      <c r="D12" t="s">
         <v>34</v>
-      </c>
-      <c r="C12" t="s">
-        <v>66</v>
-      </c>
-      <c r="D12" t="s">
-        <v>36</v>
       </c>
       <c r="E12">
         <v>2</v>
@@ -1443,21 +1446,21 @@
         <v>~$0.05</v>
       </c>
       <c r="H12" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B13" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C13" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D13" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E13">
         <v>2</v>
@@ -1470,21 +1473,21 @@
         <v>~$0.07</v>
       </c>
       <c r="H13" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B14" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C14" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D14" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E14">
         <v>10</v>
@@ -1493,25 +1496,25 @@
         <v>56</v>
       </c>
       <c r="G14" t="str">
-        <f>_xlfn.CONCAT("~$",ROUND(F14/93, 2))</f>
+        <f t="shared" ref="G14:G21" si="1">_xlfn.CONCAT("~$",ROUND(F14/93, 2))</f>
         <v>~$0.6</v>
       </c>
       <c r="H14" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B15" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C15" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D15" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E15">
         <v>2</v>
@@ -1520,22 +1523,22 @@
         <v>8</v>
       </c>
       <c r="G15" t="str">
-        <f>_xlfn.CONCAT("~$",ROUND(F15/93, 2))</f>
+        <f t="shared" si="1"/>
         <v>~$0.09</v>
       </c>
       <c r="H15" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B16" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
@@ -1547,25 +1550,25 @@
         <v>189</v>
       </c>
       <c r="G16" t="str">
-        <f>_xlfn.CONCAT("~$",ROUND(F16/93, 2))</f>
+        <f t="shared" si="1"/>
         <v>~$2.03</v>
       </c>
       <c r="H16" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" t="s">
+        <v>67</v>
+      </c>
+      <c r="C17" t="s">
+        <v>44</v>
+      </c>
+      <c r="D17" t="s">
         <v>45</v>
-      </c>
-      <c r="B17" t="s">
-        <v>69</v>
-      </c>
-      <c r="C17" t="s">
-        <v>46</v>
-      </c>
-      <c r="D17" t="s">
-        <v>47</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -1574,22 +1577,22 @@
         <v>0</v>
       </c>
       <c r="G17" t="str">
-        <f>_xlfn.CONCAT("~$",ROUND(F17/93, 2))</f>
+        <f t="shared" si="1"/>
         <v>~$0</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" t="s">
+        <v>47</v>
+      </c>
+      <c r="C18" t="s">
         <v>48</v>
       </c>
-      <c r="B18" t="s">
+      <c r="D18" t="s">
         <v>49</v>
-      </c>
-      <c r="C18" t="s">
-        <v>50</v>
-      </c>
-      <c r="D18" t="s">
-        <v>51</v>
       </c>
       <c r="E18">
         <v>70</v>
@@ -1598,25 +1601,25 @@
         <v>1680</v>
       </c>
       <c r="G18" t="str">
-        <f>_xlfn.CONCAT("~$",ROUND(F18/93, 2))</f>
+        <f t="shared" si="1"/>
         <v>~$18.06</v>
       </c>
       <c r="H18" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B19" t="s">
+        <v>51</v>
+      </c>
+      <c r="C19" t="s">
+        <v>52</v>
+      </c>
+      <c r="D19" t="s">
         <v>53</v>
-      </c>
-      <c r="C19" t="s">
-        <v>54</v>
-      </c>
-      <c r="D19" t="s">
-        <v>55</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -1625,25 +1628,25 @@
         <v>1800</v>
       </c>
       <c r="G19" t="str">
-        <f>_xlfn.CONCAT("~$",ROUND(F19/93, 2))</f>
+        <f t="shared" si="1"/>
         <v>~$19.35</v>
       </c>
       <c r="H19" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B20" t="s">
+        <v>55</v>
+      </c>
+      <c r="C20" t="s">
+        <v>56</v>
+      </c>
+      <c r="D20" t="s">
         <v>57</v>
-      </c>
-      <c r="C20" t="s">
-        <v>58</v>
-      </c>
-      <c r="D20" t="s">
-        <v>59</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -1652,24 +1655,37 @@
         <v>380</v>
       </c>
       <c r="G20" t="str">
-        <f>_xlfn.CONCAT("~$",ROUND(F20/93, 2))</f>
+        <f t="shared" si="1"/>
         <v>~$4.09</v>
       </c>
       <c r="H20" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>61</v>
+        <v>73</v>
       </c>
       <c r="F21">
-        <f>SUM(F2:F20)</f>
-        <v>10289.4</v>
+        <f>50+82+50</f>
+        <v>182</v>
       </c>
       <c r="G21" t="str">
-        <f>_xlfn.CONCAT("~$",ROUND(F21/93, 2))</f>
-        <v>~$110.64</v>
+        <f t="shared" si="1"/>
+        <v>~$1.96</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>59</v>
+      </c>
+      <c r="F22">
+        <f>SUM(F2:F21)</f>
+        <v>10619.4</v>
+      </c>
+      <c r="G22" t="str">
+        <f>_xlfn.CONCAT("~$",ROUND(F22/93, 2))</f>
+        <v>~$114.19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add printing to BOM
</commit_message>
<xml_diff>
--- a/Hardware/bom/bom.xlsx
+++ b/Hardware/bom/bom.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ritam\Documents\projects\hardware\sheaf65\Hardware\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5752D383-1FEB-4E39-B74D-F874A76BE01E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5953217A-7EC6-4546-A20A-50D56840AAC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{7EBACB66-221B-455C-9668-D99D7DBAA942}"/>
+    <workbookView xWindow="3105" yWindow="2910" windowWidth="15930" windowHeight="9165" xr2:uid="{7EBACB66-221B-455C-9668-D99D7DBAA942}"/>
   </bookViews>
   <sheets>
     <sheet name="bom" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="75">
   <si>
     <t>Category</t>
   </si>
@@ -170,9 +170,6 @@
     <t>3D printed</t>
   </si>
   <si>
-    <t>Self / Print Legion</t>
-  </si>
-  <si>
     <t>Keyboard Part</t>
   </si>
   <si>
@@ -255,6 +252,12 @@
   </si>
   <si>
     <t>Shipping</t>
+  </si>
+  <si>
+    <t>Robu.in FDM</t>
+  </si>
+  <si>
+    <t>https://robu.in/product/3d-printing-service1</t>
   </si>
 </sst>
 </file>
@@ -1295,10 +1298,10 @@
         <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E7">
         <v>68</v>
@@ -1403,7 +1406,7 @@
         <v>32</v>
       </c>
       <c r="C11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D11" t="s">
         <v>34</v>
@@ -1419,7 +1422,7 @@
         <v>~$0.47</v>
       </c>
       <c r="H11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
@@ -1430,7 +1433,7 @@
         <v>32</v>
       </c>
       <c r="C12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D12" t="s">
         <v>34</v>
@@ -1446,7 +1449,7 @@
         <v>~$0.05</v>
       </c>
       <c r="H12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
@@ -1454,10 +1457,10 @@
         <v>31</v>
       </c>
       <c r="B13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" t="s">
         <v>62</v>
-      </c>
-      <c r="C13" t="s">
-        <v>63</v>
       </c>
       <c r="D13" t="s">
         <v>34</v>
@@ -1473,7 +1476,7 @@
         <v>~$0.07</v>
       </c>
       <c r="H13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
@@ -1535,10 +1538,10 @@
         <v>43</v>
       </c>
       <c r="B16" t="s">
+        <v>67</v>
+      </c>
+      <c r="C16" t="s">
         <v>68</v>
-      </c>
-      <c r="C16" t="s">
-        <v>69</v>
       </c>
       <c r="D16" t="s">
         <v>11</v>
@@ -1554,7 +1557,7 @@
         <v>~$2.03</v>
       </c>
       <c r="H16" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
@@ -1562,37 +1565,40 @@
         <v>43</v>
       </c>
       <c r="B17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C17" t="s">
         <v>44</v>
       </c>
       <c r="D17" t="s">
-        <v>45</v>
+        <v>73</v>
       </c>
       <c r="E17">
         <v>1</v>
       </c>
       <c r="F17">
-        <v>0</v>
+        <v>990</v>
       </c>
       <c r="G17" t="str">
         <f t="shared" si="1"/>
-        <v>~$0</v>
+        <v>~$10.65</v>
+      </c>
+      <c r="H17" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" t="s">
         <v>46</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>47</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>48</v>
-      </c>
-      <c r="D18" t="s">
-        <v>49</v>
       </c>
       <c r="E18">
         <v>70</v>
@@ -1605,21 +1611,21 @@
         <v>~$18.06</v>
       </c>
       <c r="H18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B19" t="s">
+        <v>50</v>
+      </c>
+      <c r="C19" t="s">
         <v>51</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>52</v>
-      </c>
-      <c r="D19" t="s">
-        <v>53</v>
       </c>
       <c r="E19">
         <v>1</v>
@@ -1632,21 +1638,21 @@
         <v>~$19.35</v>
       </c>
       <c r="H19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B20" t="s">
+        <v>54</v>
+      </c>
+      <c r="C20" t="s">
         <v>55</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>56</v>
-      </c>
-      <c r="D20" t="s">
-        <v>57</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -1659,12 +1665,12 @@
         <v>~$4.09</v>
       </c>
       <c r="H20" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F21">
         <f>50+82+50</f>
@@ -1677,15 +1683,15 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F22">
         <f>SUM(F2:F21)</f>
-        <v>10622.4</v>
+        <v>11612.4</v>
       </c>
       <c r="G22" t="str">
         <f>_xlfn.CONCAT("~$",ROUND(F22/93, 2))</f>
-        <v>~$114.22</v>
+        <v>~$124.86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>